<commit_message>
Agrega leyenda de abreviaturas en PDF, panel HTML, Excel y NOTAS
</commit_message>
<xml_diff>
--- a/excel/04_analisis.xlsx
+++ b/excel/04_analisis.xlsx
@@ -13,7 +13,8 @@
     <sheet name="Fructosamina est." sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Laboratorio" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Bibliografia" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Notas IA" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Leyenda" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Notas IA" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -9108,6 +9109,216 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:B16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="62" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Abreviatura</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Significado</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>TIR</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Tiempo dentro del rango: % de lecturas en 100-250 mg/dL</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>TAR</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Tiempo por encima del rango: % de lecturas &gt; 250 mg/dL</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>TBR</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Tiempo por debajo del rango: % de lecturas &lt; 80 mg/dL</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>CV</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Coeficiente de variación: desviación estándar / media x 100</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>SD</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Desviación estándar</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>GLU</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Glucosa (lecturas de planillas, mg/dL)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Fructosamina (µmol/L)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>eAG</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Glucosa promedio estimada (estimated average glucose)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>CGM / BG</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Monitorización continua de glucosa / Glucosa sanguínea</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>UCCR</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Cociente cortisol-creatinina urinaria (control del Cushing)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>UPC</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Cociente proteína-creatinina urinaria (proteinuria)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>LPCE / cPLI</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Lipasa pancreática específica canina</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Hto / Hb</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Hematocrito / Hemoglobina</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>T4 libre / TSH</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Tiroxina libre / Hormona estimulante de la tiroides</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>ALT (GPT) / FAL / GGT</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Enzimas hepáticas: alanina-aminotransferasa / fosfatasa alcalina / gamma-glutamil transferasa</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>